<commit_message>
Ajuste na cor do botão
</commit_message>
<xml_diff>
--- a/src/data/Apoio_base_dashboard.xlsx
+++ b/src/data/Apoio_base_dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luiz.cagnon\Downloads\project-bolt-sb1-8qphqada\project\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C709C33D-4115-4F10-85BC-0EE5B6570829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5098E94B-5C07-44CC-9B70-AEC38F059A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D0945927-1537-4A1E-A55C-B56DE6E5501F}"/>
   </bookViews>
@@ -131,7 +131,7 @@
     <t>https://app.powerbi.com/reportEmbed?reportId=693d86a7-13bc-4ffb-b8f0-58a6c6c92a84&amp;autoAuth=true&amp;ctid=50346803-3299-4314-bb54-e86716cc07b3</t>
   </si>
   <si>
-    <t>https://app.powerbi.com/links/qWftYpVse_?ctid=50346803-3299-4314-bb54-e86716cc07b3&amp;pbi_source=linkShare&amp;bookmarkGuid=73949abc-ac85-492a-a778-e77097d10a76</t>
+    <t>https://app.powerbi.com/links/qWftYpVse_?ctid=50346803-3299-4314-bb54-e86716cc07b3&amp;pbi_source=linkShare</t>
   </si>
 </sst>
 </file>
@@ -648,13 +648,13 @@
     <hyperlink ref="C5" r:id="rId3" xr:uid="{06D255C3-110B-4699-B385-B24450426877}"/>
     <hyperlink ref="C6" r:id="rId4" xr:uid="{2C7D8C97-5396-4203-8021-F800C3292692}"/>
     <hyperlink ref="C7" r:id="rId5" display="https://app.powerbi.com/Redirect?action=OpenReport&amp;appId=f3ce25f6-a8e3-4236-b01e-ad44b68fc77f&amp;reportObjectId=693d86a7-13bc-4ffb-b8f0-58a6c6c92a84&amp;ctid=50346803-3299-4314-bb54-e86716cc07b3&amp;reportPage=c3b490991b472438a007&amp;pbi_source=appShareLink&amp;portalSessionId=7f67e39f-9e46-4446-bfc5-b4e6d501593a" xr:uid="{8F4A7C7B-5C61-426E-BE3A-CE057A7F5024}"/>
-    <hyperlink ref="E2" r:id="rId6" xr:uid="{090792EF-179A-4D51-81EB-E80007D90229}"/>
-    <hyperlink ref="E3" r:id="rId7" xr:uid="{4C1D2110-7221-4C1A-A934-15195B2987EE}"/>
-    <hyperlink ref="E4" r:id="rId8" xr:uid="{58F59087-F5D7-4F06-82DA-68A23618C438}"/>
-    <hyperlink ref="E5" r:id="rId9" xr:uid="{964BCF43-0F5E-4F76-A340-19DC64EB4FA2}"/>
-    <hyperlink ref="E6" r:id="rId10" xr:uid="{20BD58D7-2CC8-4D40-813E-8565B3BE4F52}"/>
-    <hyperlink ref="E7" r:id="rId11" xr:uid="{92E8EBA1-4231-4C96-8F59-807EDE9ECA76}"/>
-    <hyperlink ref="C2" r:id="rId12" xr:uid="{D0375E45-A245-4D2E-8EE6-A857B3112E85}"/>
+    <hyperlink ref="E3" r:id="rId6" xr:uid="{4C1D2110-7221-4C1A-A934-15195B2987EE}"/>
+    <hyperlink ref="E4" r:id="rId7" xr:uid="{58F59087-F5D7-4F06-82DA-68A23618C438}"/>
+    <hyperlink ref="E5" r:id="rId8" xr:uid="{964BCF43-0F5E-4F76-A340-19DC64EB4FA2}"/>
+    <hyperlink ref="E6" r:id="rId9" xr:uid="{20BD58D7-2CC8-4D40-813E-8565B3BE4F52}"/>
+    <hyperlink ref="E7" r:id="rId10" xr:uid="{92E8EBA1-4231-4C96-8F59-807EDE9ECA76}"/>
+    <hyperlink ref="C2" r:id="rId11" xr:uid="{9434535A-D8FB-426D-B758-4897768D69E6}"/>
+    <hyperlink ref="E2" r:id="rId12" xr:uid="{B1FD34D3-9E1D-4C0C-A7C2-76E8A8104014}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>